<commit_message>
termino inclusão da parte social e melhoramento na pagina e correção dos label critico, alto, baixo em todos os locais.
</commit_message>
<xml_diff>
--- a/etl/data/mis/1200179 - Capixaba.xlsx
+++ b/etl/data/mis/1200179 - Capixaba.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projetos\frontend\etl\data\mis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuário\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CD8107-F516-473F-B863-70065B975A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11856"/>
   </bookViews>
   <sheets>
     <sheet name="capixaba" sheetId="1" r:id="rId1"/>
@@ -57,13 +56,13 @@
     <t>IBGE - População Estimada</t>
   </si>
   <si>
-    <t>COD MUN</t>
+    <t>codigo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -376,9 +375,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K157"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="12.21875" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -4226,8 +4229,8 @@
       <c r="J110" s="2">
         <v>178375</v>
       </c>
-      <c r="K110">
-        <v>0</v>
+      <c r="K110" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
@@ -4261,8 +4264,8 @@
       <c r="J111" s="2">
         <v>182281</v>
       </c>
-      <c r="K111">
-        <v>0</v>
+      <c r="K111" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
@@ -4296,8 +4299,8 @@
       <c r="J112" s="2">
         <v>186186.70310000001</v>
       </c>
-      <c r="K112">
-        <v>0</v>
+      <c r="K112" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
@@ -4331,8 +4334,8 @@
       <c r="J113" s="2">
         <v>186186.79689999999</v>
       </c>
-      <c r="K113">
-        <v>0</v>
+      <c r="K113" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
@@ -4366,8 +4369,8 @@
       <c r="J114" s="2">
         <v>188760.79689999999</v>
       </c>
-      <c r="K114">
-        <v>0</v>
+      <c r="K114" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.3">
@@ -4401,8 +4404,8 @@
       <c r="J115" s="2">
         <v>196681.29689999999</v>
       </c>
-      <c r="K115">
-        <v>0</v>
+      <c r="K115" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.3">
@@ -4436,8 +4439,8 @@
       <c r="J116" s="2">
         <v>196681.29689999999</v>
       </c>
-      <c r="K116">
-        <v>0</v>
+      <c r="K116" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
@@ -4471,8 +4474,8 @@
       <c r="J117" s="2">
         <v>201962.07810000001</v>
       </c>
-      <c r="K117">
-        <v>0</v>
+      <c r="K117" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.3">
@@ -4506,8 +4509,8 @@
       <c r="J118" s="2">
         <v>207242.07810000001</v>
       </c>
-      <c r="K118">
-        <v>0</v>
+      <c r="K118" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
@@ -4541,8 +4544,8 @@
       <c r="J119" s="2">
         <v>205922.3438</v>
       </c>
-      <c r="K119">
-        <v>0</v>
+      <c r="K119" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.3">
@@ -4576,8 +4579,8 @@
       <c r="J120" s="2">
         <v>213846.92189999999</v>
       </c>
-      <c r="K120">
-        <v>0</v>
+      <c r="K120" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.3">
@@ -4611,8 +4614,8 @@
       <c r="J121" s="2">
         <v>219121.82810000001</v>
       </c>
-      <c r="K121">
-        <v>0</v>
+      <c r="K121" s="1">
+        <v>12280</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.3">
@@ -4643,6 +4646,9 @@
       <c r="J122" s="2">
         <v>232982.01560000001</v>
       </c>
+      <c r="K122" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123">
@@ -4672,6 +4678,9 @@
       <c r="J123" s="2">
         <v>242866.20310000001</v>
       </c>
+      <c r="K123" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124">
@@ -4701,6 +4710,9 @@
       <c r="J124" s="2">
         <v>241455.7188</v>
       </c>
+      <c r="K124" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A125">
@@ -4730,6 +4742,9 @@
       <c r="J125" s="2">
         <v>249928.4375</v>
       </c>
+      <c r="K125" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126">
@@ -4759,6 +4774,9 @@
       <c r="J126" s="2">
         <v>252754.0625</v>
       </c>
+      <c r="K126" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127">
@@ -4788,6 +4806,9 @@
       <c r="J127" s="2">
         <v>255579.9062</v>
       </c>
+      <c r="K127" s="1">
+        <v>12280</v>
+      </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A128">
@@ -4817,8 +4838,11 @@
       <c r="J128" s="2">
         <v>249958.125</v>
       </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K128" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>1200179</v>
       </c>
@@ -4846,8 +4870,11 @@
       <c r="J129" s="2">
         <v>104501.2812</v>
       </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K129" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>1200179</v>
       </c>
@@ -4875,8 +4902,11 @@
       <c r="J130" s="2">
         <v>81907.257800000007</v>
       </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K130" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>1200179</v>
       </c>
@@ -4904,8 +4934,11 @@
       <c r="J131" s="2">
         <v>81907.710900000005</v>
       </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K131" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>1200179</v>
       </c>
@@ -4933,8 +4966,11 @@
       <c r="J132" s="2">
         <v>67788.140599999999</v>
       </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K132" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>1200179</v>
       </c>
@@ -4962,8 +4998,11 @@
       <c r="J133" s="2">
         <v>63548.800799999997</v>
       </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K133" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>1200179</v>
       </c>
@@ -4991,8 +5030,11 @@
       <c r="J134" s="2">
         <v>62246.890599999999</v>
       </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K134" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>1200179</v>
       </c>
@@ -5020,8 +5062,11 @@
       <c r="J135" s="2">
         <v>62249.460899999998</v>
       </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K135" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>1200179</v>
       </c>
@@ -5049,8 +5094,11 @@
       <c r="J136" s="2">
         <v>60730.351600000002</v>
       </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K136" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>1200179</v>
       </c>
@@ -5078,8 +5126,11 @@
       <c r="J137" s="2">
         <v>60729.828099999999</v>
       </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K137" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>1200179</v>
       </c>
@@ -5107,8 +5158,11 @@
       <c r="J138" s="2">
         <v>63764.781199999998</v>
       </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K138" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>1200179</v>
       </c>
@@ -5136,8 +5190,11 @@
       <c r="J139" s="2">
         <v>69836.75</v>
       </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K139" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>1200179</v>
       </c>
@@ -5165,8 +5222,11 @@
       <c r="J140" s="2">
         <v>62246.039100000002</v>
       </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K140" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>1200179</v>
       </c>
@@ -5194,8 +5254,11 @@
       <c r="J141" s="2">
         <v>65282.25</v>
       </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K141" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>1200179</v>
       </c>
@@ -5223,8 +5286,11 @@
       <c r="J142" s="2">
         <v>59210.519500000002</v>
       </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K142" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>1200179</v>
       </c>
@@ -5252,8 +5318,11 @@
       <c r="J143" s="2">
         <v>60728.308599999997</v>
       </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K143" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>1200179</v>
       </c>
@@ -5281,8 +5350,11 @@
       <c r="J144" s="2">
         <v>57693.539100000002</v>
       </c>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K144" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>1200179</v>
       </c>
@@ -5310,8 +5382,11 @@
       <c r="J145" s="2">
         <v>54656.308599999997</v>
       </c>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K145" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>1200179</v>
       </c>
@@ -5339,8 +5414,11 @@
       <c r="J146" s="2">
         <v>56742.640599999999</v>
       </c>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K146" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>1200179</v>
       </c>
@@ -5368,8 +5446,11 @@
       <c r="J147" s="2">
         <v>53501.289100000002</v>
       </c>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K147" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>1200179</v>
       </c>
@@ -5397,8 +5478,11 @@
       <c r="J148" s="2">
         <v>58364</v>
       </c>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K148" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>1200179</v>
       </c>
@@ -5426,8 +5510,11 @@
       <c r="J149">
         <v>0</v>
       </c>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K149" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>1200179</v>
       </c>
@@ -5455,8 +5542,11 @@
       <c r="J150">
         <v>0</v>
       </c>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K150" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>1200179</v>
       </c>
@@ -5484,8 +5574,11 @@
       <c r="J151">
         <v>0</v>
       </c>
-    </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K151" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>1200179</v>
       </c>
@@ -5513,8 +5606,11 @@
       <c r="J152">
         <v>0</v>
       </c>
-    </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K152" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>1200179</v>
       </c>
@@ -5542,8 +5638,11 @@
       <c r="J153">
         <v>0</v>
       </c>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K153" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>1200179</v>
       </c>
@@ -5571,8 +5670,11 @@
       <c r="J154">
         <v>0</v>
       </c>
-    </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K154" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>1200179</v>
       </c>
@@ -5600,8 +5702,11 @@
       <c r="J155">
         <v>0</v>
       </c>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K155" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>1200179</v>
       </c>
@@ -5629,8 +5734,11 @@
       <c r="J156">
         <v>0</v>
       </c>
-    </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K156" s="1">
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>1200179</v>
       </c>
@@ -5657,6 +5765,9 @@
       </c>
       <c r="J157">
         <v>0</v>
+      </c>
+      <c r="K157" s="1">
+        <v>12280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>